<commit_message>
fix(crm): remove all emojis and format workbook with clean institutional corporate typography
</commit_message>
<xml_diff>
--- a/KTA_Executive_Marketing_CRM_Tracker.xlsx
+++ b/KTA_Executive_Marketing_CRM_Tracker.xlsx
@@ -7,12 +7,12 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="📊 Executive Dashboard" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="🎯 Lead &amp; RFQ Pipeline" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="🏨 Key Client Accounts" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="📦 Welcome Box Tracker" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="💬 WhatsApp Outreach Engine" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="🌿 Wholesale SKU Pricing" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Executive Dashboard" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lead &amp; RFQ Pipeline" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Key Client Accounts" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Welcome Box Tracker" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WhatsApp Outreach Engine" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Wholesale SKU Pricing" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -37,25 +37,19 @@
       <name val="Calibri"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="002B3917"/>
       <sz val="16"/>
     </font>
     <font>
       <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="002B3917"/>
-      <sz val="18"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <b val="1"/>
-      <color rgb="00475569"/>
-      <sz val="9"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <b val="1"/>
-      <color rgb="00FFFFFF"/>
-      <sz val="12"/>
+      <color rgb="004B5563"/>
+      <sz val="8.5"/>
     </font>
     <font>
       <name val="Calibri"/>
@@ -65,14 +59,20 @@
     </font>
     <font>
       <name val="Calibri"/>
-      <color rgb="000F172A"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
       <sz val="10"/>
     </font>
     <font>
       <name val="Calibri"/>
+      <color rgb="00111827"/>
+      <sz val="9.5"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="000F172A"/>
-      <sz val="10"/>
+      <color rgb="00111827"/>
+      <sz val="9.5"/>
     </font>
   </fonts>
   <fills count="8">
@@ -90,14 +90,14 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00F1F5F9"/>
-        <bgColor rgb="00F1F5F9"/>
+        <fgColor rgb="00F4F6F8"/>
+        <bgColor rgb="00F4F6F8"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00435128"/>
-        <bgColor rgb="00435128"/>
+        <fgColor rgb="003D4D24"/>
+        <bgColor rgb="003D4D24"/>
       </patternFill>
     </fill>
     <fill>
@@ -108,14 +108,14 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FAF8F5"/>
-        <bgColor rgb="00FAF8F5"/>
+        <fgColor rgb="00FAF9F6"/>
+        <bgColor rgb="00FAF9F6"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00C4A050"/>
-        <bgColor rgb="00C4A050"/>
+        <fgColor rgb="00BFA15F"/>
+        <bgColor rgb="00BFA15F"/>
       </patternFill>
     </fill>
   </fills>
@@ -129,16 +129,16 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="00CBD5E1"/>
+        <color rgb="00D1D5DB"/>
       </left>
       <right style="thin">
-        <color rgb="00CBD5E1"/>
+        <color rgb="00D1D5DB"/>
       </right>
       <top style="thin">
-        <color rgb="00CBD5E1"/>
+        <color rgb="00D1D5DB"/>
       </top>
       <bottom style="thin">
-        <color rgb="00CBD5E1"/>
+        <color rgb="00D1D5DB"/>
       </bottom>
     </border>
   </borders>
@@ -572,14 +572,14 @@
     <col width="20" customWidth="1" min="4" max="4"/>
     <col width="31" customWidth="1" min="5" max="5"/>
     <col width="28" customWidth="1" min="6" max="6"/>
-    <col width="33" customWidth="1" min="7" max="7"/>
+    <col width="31" customWidth="1" min="7" max="7"/>
     <col width="14" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>KTA SPICES — EXECUTIVE B2B MARKETING &amp; SALES CRM DASHBOARD</t>
+          <t>KOTTAYAR TRADING AGENCY — EXECUTIVE B2B MARKETING &amp; SALES CRM DASHBOARD</t>
         </is>
       </c>
     </row>
@@ -588,7 +588,7 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>₹ 48.5 Lakhs</t>
+          <t>INR 48.5 Lakhs</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
@@ -598,12 +598,12 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>42 Hotels</t>
+          <t>42 Accounts</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>34.2 %</t>
+          <t>34.2%</t>
         </is>
       </c>
     </row>
@@ -611,7 +611,7 @@
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>ACTIVE MONTHLY PIPELINE</t>
+          <t>ACTIVE MONTHLY PIPELINE VALUE</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
@@ -626,7 +626,7 @@
       </c>
       <c r="G6" s="3" t="inlineStr">
         <is>
-          <t>INBOUND RFQ TO WIN CONVERSION</t>
+          <t>INBOUND RFQ CONVERSION RATE</t>
         </is>
       </c>
     </row>
@@ -672,7 +672,7 @@
       </c>
       <c r="G10" s="5" t="inlineStr">
         <is>
-          <t>Monthly GMV (₹)</t>
+          <t>Monthly GMV (INR)</t>
         </is>
       </c>
       <c r="H10" s="5" t="inlineStr">
@@ -927,7 +927,7 @@
     <col width="22" customWidth="1" min="8" max="8"/>
     <col width="48" customWidth="1" min="9" max="9"/>
     <col width="17" customWidth="1" min="10" max="10"/>
-    <col width="18" customWidth="1" min="11" max="11"/>
+    <col width="20" customWidth="1" min="11" max="11"/>
     <col width="21" customWidth="1" min="12" max="12"/>
     <col width="48" customWidth="1" min="13" max="13"/>
   </cols>
@@ -935,7 +935,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>KTA SPICES — INBOUND COMMERCIAL LEADS &amp; SAMPLE RFQ PIPELINE</t>
+          <t>INBOUND COMMERCIAL LEADS &amp; SAMPLE RFQ PIPELINE</t>
         </is>
       </c>
     </row>
@@ -992,7 +992,7 @@
       </c>
       <c r="K2" s="5" t="inlineStr">
         <is>
-          <t>Deal Value (₹)</t>
+          <t>Deal Value (INR)</t>
         </is>
       </c>
       <c r="L2" s="5" t="inlineStr">
@@ -1474,13 +1474,13 @@
     <col width="21" customWidth="1" min="8" max="8"/>
     <col width="45" customWidth="1" min="9" max="9"/>
     <col width="36" customWidth="1" min="10" max="10"/>
-    <col width="23" customWidth="1" min="11" max="11"/>
+    <col width="25" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>KTA SPICES — KEY HOTEL &amp; COMMERCIAL KITCHEN ACCOUNTS DIRECTORY</t>
+          <t>KEY HOTEL &amp; COMMERCIAL KITCHEN ACCOUNTS DIRECTORY</t>
         </is>
       </c>
     </row>
@@ -1537,7 +1537,7 @@
       </c>
       <c r="K2" s="5" t="inlineStr">
         <is>
-          <t>Annual Run-Rate (₹)</t>
+          <t>Annual Run-Rate (INR)</t>
         </is>
       </c>
     </row>
@@ -1884,14 +1884,14 @@
     <col width="22" customWidth="1" min="6" max="6"/>
     <col width="19" customWidth="1" min="7" max="7"/>
     <col width="26" customWidth="1" min="8" max="8"/>
-    <col width="23" customWidth="1" min="9" max="9"/>
-    <col width="24" customWidth="1" min="10" max="10"/>
+    <col width="22" customWidth="1" min="9" max="9"/>
+    <col width="26" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>KTA SPICES — CHEF WELCOME BOX &amp; DISCOVERY SAMPLE KIT DISPATCH LOG</t>
+          <t>CHEF WELCOME BOX &amp; DISCOVERY SAMPLE KIT DISPATCH LOG</t>
         </is>
       </c>
     </row>
@@ -1938,12 +1938,12 @@
       </c>
       <c r="I2" s="5" t="inlineStr">
         <is>
-          <t>Converted to Order?</t>
+          <t>Converted to Order</t>
         </is>
       </c>
       <c r="J2" s="5" t="inlineStr">
         <is>
-          <t>Initial PO Value (₹)</t>
+          <t>Initial PO Value (INR)</t>
         </is>
       </c>
     </row>
@@ -1985,7 +1985,7 @@
       </c>
       <c r="H3" s="7" t="inlineStr">
         <is>
-          <t>⭐⭐⭐⭐⭐ (5/5)</t>
+          <t>5.0 / 5.0 (Approved)</t>
         </is>
       </c>
       <c r="I3" s="7" t="inlineStr">
@@ -2035,7 +2035,7 @@
       </c>
       <c r="H4" s="11" t="inlineStr">
         <is>
-          <t>⭐⭐⭐⭐⭐ (5/5)</t>
+          <t>5.0 / 5.0 (Approved)</t>
         </is>
       </c>
       <c r="I4" s="11" t="inlineStr">
@@ -2085,7 +2085,7 @@
       </c>
       <c r="H5" s="7" t="inlineStr">
         <is>
-          <t>⭐⭐⭐⭐ (4/5)</t>
+          <t>4.5 / 5.0 (Approved)</t>
         </is>
       </c>
       <c r="I5" s="7" t="inlineStr">
@@ -2135,7 +2135,7 @@
       </c>
       <c r="H6" s="11" t="inlineStr">
         <is>
-          <t>⭐⭐⭐⭐⭐ (5/5)</t>
+          <t>4.8 / 5.0 (Approved)</t>
         </is>
       </c>
       <c r="I6" s="11" t="inlineStr">
@@ -2185,7 +2185,7 @@
       </c>
       <c r="H7" s="7" t="inlineStr">
         <is>
-          <t>Evaluating</t>
+          <t>In Evaluation</t>
         </is>
       </c>
       <c r="I7" s="7" t="inlineStr">
@@ -2222,13 +2222,13 @@
     <col width="20" customWidth="1" min="6" max="6"/>
     <col width="16" customWidth="1" min="7" max="7"/>
     <col width="18" customWidth="1" min="8" max="8"/>
-    <col width="22" customWidth="1" min="9" max="9"/>
+    <col width="24" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>KTA SPICES — WHATSAPP B2B CAMPAIGN &amp; PRO-FORMA CONVERSION LOG</t>
+          <t>WHATSAPP B2B CAMPAIGN &amp; PRO-FORMA CONVERSION LOG</t>
         </is>
       </c>
     </row>
@@ -2275,7 +2275,7 @@
       </c>
       <c r="I2" s="5" t="inlineStr">
         <is>
-          <t>Closed Revenue (₹)</t>
+          <t>Closed Revenue (INR)</t>
         </is>
       </c>
     </row>
@@ -2452,14 +2452,14 @@
   <dimension ref="A1:J12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="48" customWidth="1" min="1" max="1"/>
+    <col width="44" customWidth="1" min="1" max="1"/>
     <col width="48" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="21" customWidth="1" min="4" max="4"/>
-    <col width="25" customWidth="1" min="5" max="5"/>
-    <col width="29" customWidth="1" min="6" max="6"/>
-    <col width="27" customWidth="1" min="7" max="7"/>
-    <col width="24" customWidth="1" min="8" max="8"/>
+    <col width="27" customWidth="1" min="5" max="5"/>
+    <col width="31" customWidth="1" min="6" max="6"/>
+    <col width="29" customWidth="1" min="7" max="7"/>
+    <col width="26" customWidth="1" min="8" max="8"/>
     <col width="18" customWidth="1" min="9" max="9"/>
     <col width="47" customWidth="1" min="10" max="10"/>
   </cols>
@@ -2467,7 +2467,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>KTA SPICES — WHOLESALE SKU PRICE, MOQ &amp; MARGIN MATRIX</t>
+          <t>WHOLESALE SKU PRICE, MOQ &amp; MARGIN MATRIX</t>
         </is>
       </c>
     </row>
@@ -2494,22 +2494,22 @@
       </c>
       <c r="E2" s="5" t="inlineStr">
         <is>
-          <t>Farm-Gate Cost (₹/kg)</t>
+          <t>Farm-Gate Cost (INR/kg)</t>
         </is>
       </c>
       <c r="F2" s="5" t="inlineStr">
         <is>
-          <t>Freight &amp; Cleaning (₹/kg)</t>
+          <t>Freight &amp; Cleaning (INR/kg)</t>
         </is>
       </c>
       <c r="G2" s="5" t="inlineStr">
         <is>
-          <t>Wholesale 500kg+ (₹/kg)</t>
+          <t>Wholesale 500kg+ (INR/kg)</t>
         </is>
       </c>
       <c r="H2" s="5" t="inlineStr">
         <is>
-          <t>Multi-Ton 2T+ (₹/kg)</t>
+          <t>Multi-Ton 2T+ (INR/kg)</t>
         </is>
       </c>
       <c r="I2" s="5" t="inlineStr">

</xml_diff>

<commit_message>
feat(crm): expand workbook with manager operations log, weekly/monthly management reports, warehouse QC inventory, and dispatch invoicing ledger
</commit_message>
<xml_diff>
--- a/KTA_Executive_Marketing_CRM_Tracker.xlsx
+++ b/KTA_Executive_Marketing_CRM_Tracker.xlsx
@@ -8,11 +8,14 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Executive Dashboard" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lead &amp; RFQ Pipeline" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Key Client Accounts" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Welcome Box Tracker" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WhatsApp Outreach Engine" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Wholesale SKU Pricing" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Manager Operations Log" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Management Reports" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lead &amp; RFQ Pipeline" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Key Client Accounts" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Warehouse Inventory &amp; QC" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Consignment Dispatch Log" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Welcome Box Tracker" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Wholesale SKU Pricing" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -37,42 +40,42 @@
       <name val="Calibri"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
-      <sz val="14"/>
+      <sz val="13"/>
     </font>
     <font>
       <name val="Calibri"/>
       <b val="1"/>
       <color rgb="002B3917"/>
-      <sz val="16"/>
+      <sz val="15"/>
     </font>
     <font>
       <name val="Calibri"/>
       <b val="1"/>
       <color rgb="004B5563"/>
-      <sz val="8.5"/>
+      <sz val="8"/>
     </font>
     <font>
       <name val="Calibri"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
-      <sz val="11"/>
+      <sz val="10.5"/>
     </font>
     <font>
       <name val="Calibri"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
-      <sz val="10"/>
+      <sz val="9.5"/>
     </font>
     <font>
       <name val="Calibri"/>
       <color rgb="00111827"/>
-      <sz val="9.5"/>
+      <sz val="9"/>
     </font>
     <font>
       <name val="Calibri"/>
       <b val="1"/>
       <color rgb="00111827"/>
-      <sz val="9.5"/>
+      <sz val="9"/>
     </font>
   </fonts>
   <fills count="8">
@@ -568,18 +571,18 @@
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
     <col width="19" customWidth="1" min="2" max="2"/>
-    <col width="35" customWidth="1" min="3" max="3"/>
+    <col width="31" customWidth="1" min="3" max="3"/>
     <col width="20" customWidth="1" min="4" max="4"/>
-    <col width="31" customWidth="1" min="5" max="5"/>
+    <col width="30" customWidth="1" min="5" max="5"/>
     <col width="28" customWidth="1" min="6" max="6"/>
-    <col width="31" customWidth="1" min="7" max="7"/>
+    <col width="32" customWidth="1" min="7" max="7"/>
     <col width="14" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>KOTTAYAR TRADING AGENCY — EXECUTIVE B2B MARKETING &amp; SALES CRM DASHBOARD</t>
+          <t>KOTTAYAR TRADING AGENCY — EXECUTIVE MANAGEMENT &amp; REVENUE CONTROL DASHBOARD</t>
         </is>
       </c>
     </row>
@@ -588,22 +591,22 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>INR 48.5 Lakhs</t>
+          <t>INR 3.22 Cr</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>28.4 Tons</t>
+          <t>48.8 Tons</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>42 Accounts</t>
+          <t>52 Kitchens</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>34.2%</t>
+          <t>17.4%</t>
         </is>
       </c>
     </row>
@@ -611,22 +614,22 @@
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>ACTIVE MONTHLY PIPELINE VALUE</t>
+          <t>ANNUALIZED REVENUE RUN-RATE</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>MONTHLY BULK COMMODITY RUN-RATE</t>
+          <t>TOTAL MONTHLY TRADED VOLUME</t>
         </is>
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>HOTEL SMART ACCOUNTS SERVED</t>
+          <t>ACTIVE COMMERCIAL ACCOUNTS</t>
         </is>
       </c>
       <c r="G6" s="3" t="inlineStr">
         <is>
-          <t>INBOUND RFQ CONVERSION RATE</t>
+          <t>AVERAGE BLENDED GROSS MARGIN</t>
         </is>
       </c>
     </row>
@@ -909,6 +912,839 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:K9"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="48" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="34" customWidth="1" min="3" max="3"/>
+    <col width="38" customWidth="1" min="4" max="4"/>
+    <col width="34" customWidth="1" min="5" max="5"/>
+    <col width="41" customWidth="1" min="6" max="6"/>
+    <col width="48" customWidth="1" min="7" max="7"/>
+    <col width="48" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="19" customWidth="1" min="10" max="10"/>
+    <col width="21" customWidth="1" min="11" max="11"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>TRADE DESK &amp; WAREHOUSE MANAGER DAILY OPERATIONS &amp; ACTIVITY TRACKER</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="5" t="inlineStr">
+        <is>
+          <t>Log ID</t>
+        </is>
+      </c>
+      <c r="B2" s="5" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="C2" s="5" t="inlineStr">
+        <is>
+          <t>Managing Officer</t>
+        </is>
+      </c>
+      <c r="D2" s="5" t="inlineStr">
+        <is>
+          <t>Activity Type</t>
+        </is>
+      </c>
+      <c r="E2" s="5" t="inlineStr">
+        <is>
+          <t>Target Client / Supplier / Bay</t>
+        </is>
+      </c>
+      <c r="F2" s="5" t="inlineStr">
+        <is>
+          <t>Specific Sourcing Variety</t>
+        </is>
+      </c>
+      <c r="G2" s="5" t="inlineStr">
+        <is>
+          <t>Summary &amp; Notes</t>
+        </is>
+      </c>
+      <c r="H2" s="5" t="inlineStr">
+        <is>
+          <t>Assigned Action Items</t>
+        </is>
+      </c>
+      <c r="I2" s="5" t="inlineStr">
+        <is>
+          <t>Priority</t>
+        </is>
+      </c>
+      <c r="J2" s="5" t="inlineStr">
+        <is>
+          <t>Target Deadline</t>
+        </is>
+      </c>
+      <c r="K2" s="5" t="inlineStr">
+        <is>
+          <t>Resolution Status</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="7" t="inlineStr">
+        <is>
+          <t>OPS-2026-001</t>
+        </is>
+      </c>
+      <c r="B3" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="C3" s="6" t="inlineStr">
+        <is>
+          <t>Nazeer Ahmed (Trade Desk Lead)</t>
+        </is>
+      </c>
+      <c r="D3" s="6" t="inlineStr">
+        <is>
+          <t>Client Contract Finalization</t>
+        </is>
+      </c>
+      <c r="E3" s="6" t="inlineStr">
+        <is>
+          <t>Copper Kitchen Central Prep</t>
+        </is>
+      </c>
+      <c r="F3" s="6" t="inlineStr">
+        <is>
+          <t>Tellicherry Black Pepper, Cloves</t>
+        </is>
+      </c>
+      <c r="G3" s="6" t="inlineStr">
+        <is>
+          <t>Confirmed 500kg monthly procurement schedule with Executive Chef.</t>
+        </is>
+      </c>
+      <c r="H3" s="6" t="inlineStr">
+        <is>
+          <t>Issue formal pro-forma invoice and dispatch first consignment lot.</t>
+        </is>
+      </c>
+      <c r="I3" s="7" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J3" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="K3" s="7" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="11" t="inlineStr">
+        <is>
+          <t>OPS-2026-002</t>
+        </is>
+      </c>
+      <c r="B4" s="11" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="C4" s="10" t="inlineStr">
+        <is>
+          <t>K. Sundar (Warehouse Manager)</t>
+        </is>
+      </c>
+      <c r="D4" s="10" t="inlineStr">
+        <is>
+          <t>Batch QC Assay Inspection</t>
+        </is>
+      </c>
+      <c r="E4" s="10" t="inlineStr">
+        <is>
+          <t>Mannadi Bay 2 Receiving</t>
+        </is>
+      </c>
+      <c r="F4" s="10" t="inlineStr">
+        <is>
+          <t>Alleppey Green Cardamom 8mm</t>
+        </is>
+      </c>
+      <c r="G4" s="10" t="inlineStr">
+        <is>
+          <t>Tested 25kg vacuum canisters for moisture and essential oil yield (&gt;8.5%).</t>
+        </is>
+      </c>
+      <c r="H4" s="10" t="inlineStr">
+        <is>
+          <t>Attach FSSAI batch analysis certificate to outbound consignment.</t>
+        </is>
+      </c>
+      <c r="I4" s="11" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="J4" s="11" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
+      </c>
+      <c r="K4" s="11" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="7" t="inlineStr">
+        <is>
+          <t>OPS-2026-003</t>
+        </is>
+      </c>
+      <c r="B5" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
+      </c>
+      <c r="C5" s="6" t="inlineStr">
+        <is>
+          <t>Nazeer Ahmed (Trade Desk Lead)</t>
+        </is>
+      </c>
+      <c r="D5" s="6" t="inlineStr">
+        <is>
+          <t>Executive Chef Sample Tasting</t>
+        </is>
+      </c>
+      <c r="E5" s="6" t="inlineStr">
+        <is>
+          <t>The Leela Palace Chennai</t>
+        </is>
+      </c>
+      <c r="F5" s="6" t="inlineStr">
+        <is>
+          <t>Star Anise, Cassia Bark, White Pepper</t>
+        </is>
+      </c>
+      <c r="G5" s="6" t="inlineStr">
+        <is>
+          <t>Delivered Chef Discovery Box. Chef praised aroma density and zero-polish purity.</t>
+        </is>
+      </c>
+      <c r="H5" s="6" t="inlineStr">
+        <is>
+          <t>Schedule follow-up meeting with Materials Manager for annual rates.</t>
+        </is>
+      </c>
+      <c r="I5" s="7" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J5" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="K5" s="7" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="11" t="inlineStr">
+        <is>
+          <t>OPS-2026-004</t>
+        </is>
+      </c>
+      <c r="B6" s="11" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
+      </c>
+      <c r="C6" s="10" t="inlineStr">
+        <is>
+          <t>R. Balaji (Procurement Lead)</t>
+        </is>
+      </c>
+      <c r="D6" s="10" t="inlineStr">
+        <is>
+          <t>Grower Lot Negotiations ex-Origin</t>
+        </is>
+      </c>
+      <c r="E6" s="10" t="inlineStr">
+        <is>
+          <t>Wayanad Highland Estate Group</t>
+        </is>
+      </c>
+      <c r="F6" s="10" t="inlineStr">
+        <is>
+          <t>TGSEB Black Pepper, Unbleached Ginger</t>
+        </is>
+      </c>
+      <c r="G6" s="10" t="inlineStr">
+        <is>
+          <t>Agreed forward procurement terms for 15-ton seasonal flush arrival.</t>
+        </is>
+      </c>
+      <c r="H6" s="10" t="inlineStr">
+        <is>
+          <t>Lock consignment price at INR 620/kg and confirm logistics transport.</t>
+        </is>
+      </c>
+      <c r="I6" s="11" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J6" s="11" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="K6" s="11" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="7" t="inlineStr">
+        <is>
+          <t>OPS-2026-005</t>
+        </is>
+      </c>
+      <c r="B7" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="C7" s="6" t="inlineStr">
+        <is>
+          <t>K. Sundar (Warehouse Manager)</t>
+        </is>
+      </c>
+      <c r="D7" s="6" t="inlineStr">
+        <is>
+          <t>Inventory Restock &amp; Pallet Audit</t>
+        </is>
+      </c>
+      <c r="E7" s="6" t="inlineStr">
+        <is>
+          <t>Mannadi Warehouse Bay 1</t>
+        </is>
+      </c>
+      <c r="F7" s="6" t="inlineStr">
+        <is>
+          <t>Salem Turmeric Powder (5% Curcumin)</t>
+        </is>
+      </c>
+      <c r="G7" s="6" t="inlineStr">
+        <is>
+          <t>Audited 120 master multi-wall bags (3,000kg). Sealed liner integrity verified.</t>
+        </is>
+      </c>
+      <c r="H7" s="6" t="inlineStr">
+        <is>
+          <t>Update warehouse stock ledger and reserve 1,200kg for Thalappakatti.</t>
+        </is>
+      </c>
+      <c r="I7" s="7" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="J7" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="K7" s="7" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="11" t="inlineStr">
+        <is>
+          <t>OPS-2026-006</t>
+        </is>
+      </c>
+      <c r="B8" s="11" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="C8" s="10" t="inlineStr">
+        <is>
+          <t>Nazeer Ahmed (Trade Desk Lead)</t>
+        </is>
+      </c>
+      <c r="D8" s="10" t="inlineStr">
+        <is>
+          <t>Payment Reconciliation &amp; Review</t>
+        </is>
+      </c>
+      <c r="E8" s="10" t="inlineStr">
+        <is>
+          <t>Palmshore Multi-Outlet Chain</t>
+        </is>
+      </c>
+      <c r="F8" s="10" t="inlineStr">
+        <is>
+          <t>Mixed Spice Consignment</t>
+        </is>
+      </c>
+      <c r="G8" s="10" t="inlineStr">
+        <is>
+          <t>Reconciled Invoice KTA-INV-2026-44. Payment of INR 3,85,000 received via NEFT.</t>
+        </is>
+      </c>
+      <c r="H8" s="10" t="inlineStr">
+        <is>
+          <t>Issue payment acknowledgement and update client credit ledger.</t>
+        </is>
+      </c>
+      <c r="I8" s="11" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="J8" s="11" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="K8" s="11" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="7" t="inlineStr">
+        <is>
+          <t>OPS-2026-007</t>
+        </is>
+      </c>
+      <c r="B9" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="C9" s="6" t="inlineStr">
+        <is>
+          <t>R. Balaji (Procurement Lead)</t>
+        </is>
+      </c>
+      <c r="D9" s="6" t="inlineStr">
+        <is>
+          <t>Industrial Extraction Lot Sourcing</t>
+        </is>
+      </c>
+      <c r="E9" s="6" t="inlineStr">
+        <is>
+          <t>Southern Spice Oleoresin Labs</t>
+        </is>
+      </c>
+      <c r="F9" s="6" t="inlineStr">
+        <is>
+          <t>Pinheads &amp; Lite Berries</t>
+        </is>
+      </c>
+      <c r="G9" s="6" t="inlineStr">
+        <is>
+          <t>Submitted lab assay with 6.2% piperine concentration for 5-ton extraction lot.</t>
+        </is>
+      </c>
+      <c r="H9" s="6" t="inlineStr">
+        <is>
+          <t>Receive purchase order and coordinate direct container dispatch ex-Cochin.</t>
+        </is>
+      </c>
+      <c r="I9" s="7" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J9" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="K9" s="7" t="inlineStr">
+        <is>
+          <t>Pending PO</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:K1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:L7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="48" customWidth="1" min="1" max="1"/>
+    <col width="27" customWidth="1" min="2" max="2"/>
+    <col width="21" customWidth="1" min="3" max="3"/>
+    <col width="23" customWidth="1" min="4" max="4"/>
+    <col width="28" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="23" customWidth="1" min="8" max="8"/>
+    <col width="31" customWidth="1" min="9" max="9"/>
+    <col width="27" customWidth="1" min="10" max="10"/>
+    <col width="40" customWidth="1" min="11" max="11"/>
+    <col width="48" customWidth="1" min="12" max="12"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>EXECUTIVE WEEKLY &amp; MONTHLY COMMERCIAL OPERATIONS REPORT</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="5" t="inlineStr">
+        <is>
+          <t>Period</t>
+        </is>
+      </c>
+      <c r="B2" s="5" t="inlineStr">
+        <is>
+          <t>Consignments Dispatched</t>
+        </is>
+      </c>
+      <c r="C2" s="5" t="inlineStr">
+        <is>
+          <t>Gross Volume (kg)</t>
+        </is>
+      </c>
+      <c r="D2" s="5" t="inlineStr">
+        <is>
+          <t>Gross Revenue (INR)</t>
+        </is>
+      </c>
+      <c r="E2" s="5" t="inlineStr">
+        <is>
+          <t>Cost of Goods Sold (INR)</t>
+        </is>
+      </c>
+      <c r="F2" s="5" t="inlineStr">
+        <is>
+          <t>Gross Margin (INR)</t>
+        </is>
+      </c>
+      <c r="G2" s="5" t="inlineStr">
+        <is>
+          <t>Gross Margin %</t>
+        </is>
+      </c>
+      <c r="H2" s="5" t="inlineStr">
+        <is>
+          <t>New Accounts Signed</t>
+        </is>
+      </c>
+      <c r="I2" s="5" t="inlineStr">
+        <is>
+          <t>Chef Sample Kits Dispatched</t>
+        </is>
+      </c>
+      <c r="J2" s="5" t="inlineStr">
+        <is>
+          <t>Logistics On-Time SLA %</t>
+        </is>
+      </c>
+      <c r="K2" s="5" t="inlineStr">
+        <is>
+          <t>Key Sourcing Highlight</t>
+        </is>
+      </c>
+      <c r="L2" s="5" t="inlineStr">
+        <is>
+          <t>Manager Remarks &amp; Corrective Measures</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="7" t="inlineStr">
+        <is>
+          <t>Week 31 (Aug 1 - Aug 7)</t>
+        </is>
+      </c>
+      <c r="B3" s="6" t="n">
+        <v>24</v>
+      </c>
+      <c r="C3" s="8" t="n">
+        <v>11200</v>
+      </c>
+      <c r="D3" s="9" t="n">
+        <v>7420000</v>
+      </c>
+      <c r="E3" s="9" t="n">
+        <v>6140000</v>
+      </c>
+      <c r="F3" s="9" t="n">
+        <v>1280000</v>
+      </c>
+      <c r="G3" s="7" t="inlineStr">
+        <is>
+          <t>17.3%</t>
+        </is>
+      </c>
+      <c r="H3" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="I3" s="7" t="n">
+        <v>14</v>
+      </c>
+      <c r="J3" s="7" t="inlineStr">
+        <is>
+          <t>98.5%</t>
+        </is>
+      </c>
+      <c r="K3" s="6" t="inlineStr">
+        <is>
+          <t>Pepper export bold demand high</t>
+        </is>
+      </c>
+      <c r="L3" s="6" t="inlineStr">
+        <is>
+          <t>Achieved zero transit delay across Chennai central kitchen deliveries.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="11" t="inlineStr">
+        <is>
+          <t>Week 32 (Aug 8 - Aug 14)</t>
+        </is>
+      </c>
+      <c r="B4" s="10" t="n">
+        <v>28</v>
+      </c>
+      <c r="C4" s="12" t="n">
+        <v>12800</v>
+      </c>
+      <c r="D4" s="13" t="n">
+        <v>8460000</v>
+      </c>
+      <c r="E4" s="13" t="n">
+        <v>6980000</v>
+      </c>
+      <c r="F4" s="13" t="n">
+        <v>1480000</v>
+      </c>
+      <c r="G4" s="11" t="inlineStr">
+        <is>
+          <t>17.5%</t>
+        </is>
+      </c>
+      <c r="H4" s="11" t="n">
+        <v>4</v>
+      </c>
+      <c r="I4" s="11" t="n">
+        <v>18</v>
+      </c>
+      <c r="J4" s="11" t="inlineStr">
+        <is>
+          <t>99.0%</t>
+        </is>
+      </c>
+      <c r="K4" s="10" t="inlineStr">
+        <is>
+          <t>Cardamom 8mm flush arrivals secured</t>
+        </is>
+      </c>
+      <c r="L4" s="10" t="inlineStr">
+        <is>
+          <t>Expanded Hotel Smart delivery routes to cover OMR and Guindy hospitality belts.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="7" t="inlineStr">
+        <is>
+          <t>Week 33 (Aug 15 - Aug 21)</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="n">
+        <v>26</v>
+      </c>
+      <c r="C5" s="8" t="n">
+        <v>11900</v>
+      </c>
+      <c r="D5" s="9" t="n">
+        <v>7890000</v>
+      </c>
+      <c r="E5" s="9" t="n">
+        <v>6520000</v>
+      </c>
+      <c r="F5" s="9" t="n">
+        <v>1370000</v>
+      </c>
+      <c r="G5" s="7" t="inlineStr">
+        <is>
+          <t>17.4%</t>
+        </is>
+      </c>
+      <c r="H5" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="I5" s="7" t="n">
+        <v>16</v>
+      </c>
+      <c r="J5" s="7" t="inlineStr">
+        <is>
+          <t>97.8%</t>
+        </is>
+      </c>
+      <c r="K5" s="6" t="inlineStr">
+        <is>
+          <t>Dry ginger Cochin unbleached steady</t>
+        </is>
+      </c>
+      <c r="L5" s="6" t="inlineStr">
+        <is>
+          <t>Secured additional buffer stock in Mannadi to safeguard banquet festival peaks.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="11" t="inlineStr">
+        <is>
+          <t>Week 34 (Aug 22 - Aug 28)</t>
+        </is>
+      </c>
+      <c r="B6" s="10" t="n">
+        <v>31</v>
+      </c>
+      <c r="C6" s="12" t="n">
+        <v>12900</v>
+      </c>
+      <c r="D6" s="13" t="n">
+        <v>8464000</v>
+      </c>
+      <c r="E6" s="13" t="n">
+        <v>6984000</v>
+      </c>
+      <c r="F6" s="13" t="n">
+        <v>1480000</v>
+      </c>
+      <c r="G6" s="11" t="inlineStr">
+        <is>
+          <t>17.5%</t>
+        </is>
+      </c>
+      <c r="H6" s="11" t="n">
+        <v>5</v>
+      </c>
+      <c r="I6" s="11" t="n">
+        <v>22</v>
+      </c>
+      <c r="J6" s="11" t="inlineStr">
+        <is>
+          <t>99.2%</t>
+        </is>
+      </c>
+      <c r="K6" s="10" t="inlineStr">
+        <is>
+          <t>Record welcome sample box conversion</t>
+        </is>
+      </c>
+      <c r="L6" s="10" t="inlineStr">
+        <is>
+          <t>Signed multi-outlet annual agreement with Copper Kitchen &amp; Buhari establishments.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="15" t="inlineStr">
+        <is>
+          <t>MONTHLY TOTAL (AUGUST 2026)</t>
+        </is>
+      </c>
+      <c r="B7" s="14" t="n">
+        <v>109</v>
+      </c>
+      <c r="C7" s="16" t="n">
+        <v>48800</v>
+      </c>
+      <c r="D7" s="17" t="n">
+        <v>32234000</v>
+      </c>
+      <c r="E7" s="17" t="n">
+        <v>26624000</v>
+      </c>
+      <c r="F7" s="17" t="n">
+        <v>5610000</v>
+      </c>
+      <c r="G7" s="15" t="inlineStr">
+        <is>
+          <t>17.4%</t>
+        </is>
+      </c>
+      <c r="H7" s="15" t="n">
+        <v>14</v>
+      </c>
+      <c r="I7" s="15" t="n">
+        <v>70</v>
+      </c>
+      <c r="J7" s="15" t="inlineStr">
+        <is>
+          <t>98.6%</t>
+        </is>
+      </c>
+      <c r="K7" s="14" t="inlineStr">
+        <is>
+          <t>Strong institutional momentum</t>
+        </is>
+      </c>
+      <c r="L7" s="14" t="inlineStr">
+        <is>
+          <t>Surpassed monthly revenue target by 14.8%. Working capital cycle at 18 days.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:L1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -935,7 +1771,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>INBOUND COMMERCIAL LEADS &amp; SAMPLE RFQ PIPELINE</t>
+          <t>INBOUND COMMERCIAL LEADS &amp; SAMPLE RFQ PIPELINE (WITH MANAGER CONTROLS)</t>
         </is>
       </c>
     </row>
@@ -1455,7 +2291,894 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:L8"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="48" customWidth="1" min="1" max="1"/>
+    <col width="34" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="24" customWidth="1" min="5" max="5"/>
+    <col width="19" customWidth="1" min="6" max="6"/>
+    <col width="21" customWidth="1" min="7" max="7"/>
+    <col width="45" customWidth="1" min="8" max="8"/>
+    <col width="18" customWidth="1" min="9" max="9"/>
+    <col width="18" customWidth="1" min="10" max="10"/>
+    <col width="19" customWidth="1" min="11" max="11"/>
+    <col width="25" customWidth="1" min="12" max="12"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>KEY COMMERCIAL ACCOUNTS &amp; OUTSTANDING FINANCIAL CONTROL LEDGER</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="5" t="inlineStr">
+        <is>
+          <t>Account Code</t>
+        </is>
+      </c>
+      <c r="B2" s="5" t="inlineStr">
+        <is>
+          <t>Property / Enterprise Name</t>
+        </is>
+      </c>
+      <c r="C2" s="5" t="inlineStr">
+        <is>
+          <t>Establishment Tier</t>
+        </is>
+      </c>
+      <c r="D2" s="5" t="inlineStr">
+        <is>
+          <t>City / Destination</t>
+        </is>
+      </c>
+      <c r="E2" s="5" t="inlineStr">
+        <is>
+          <t>Chef / Purchase Lead</t>
+        </is>
+      </c>
+      <c r="F2" s="5" t="inlineStr">
+        <is>
+          <t>Direct Mobile</t>
+        </is>
+      </c>
+      <c r="G2" s="5" t="inlineStr">
+        <is>
+          <t>Monthly Vol. (kg)</t>
+        </is>
+      </c>
+      <c r="H2" s="5" t="inlineStr">
+        <is>
+          <t>Key SKUs Sourced</t>
+        </is>
+      </c>
+      <c r="I2" s="5" t="inlineStr">
+        <is>
+          <t>Credit Terms</t>
+        </is>
+      </c>
+      <c r="J2" s="5" t="inlineStr">
+        <is>
+          <t>Payment Status</t>
+        </is>
+      </c>
+      <c r="K2" s="5" t="inlineStr">
+        <is>
+          <t>Outstanding INR</t>
+        </is>
+      </c>
+      <c r="L2" s="5" t="inlineStr">
+        <is>
+          <t>Annual Run-Rate (INR)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="7" t="inlineStr">
+        <is>
+          <t>KTA-ACC-01</t>
+        </is>
+      </c>
+      <c r="B3" s="6" t="inlineStr">
+        <is>
+          <t>Copper Kitchen Multi-Outlet</t>
+        </is>
+      </c>
+      <c r="C3" s="7" t="inlineStr">
+        <is>
+          <t>Premium Casual Chain (8 Outlets)</t>
+        </is>
+      </c>
+      <c r="D3" s="6" t="inlineStr">
+        <is>
+          <t>Chennai, TN</t>
+        </is>
+      </c>
+      <c r="E3" s="6" t="inlineStr">
+        <is>
+          <t>Chef Arshad</t>
+        </is>
+      </c>
+      <c r="F3" s="7" t="inlineStr">
+        <is>
+          <t>+91 85928 32871</t>
+        </is>
+      </c>
+      <c r="G3" s="8" t="n">
+        <v>1200</v>
+      </c>
+      <c r="H3" s="6" t="inlineStr">
+        <is>
+          <t>Black Pepper, Kashmiri Chilli, Cloves</t>
+        </is>
+      </c>
+      <c r="I3" s="7" t="inlineStr">
+        <is>
+          <t>15 Days Net</t>
+        </is>
+      </c>
+      <c r="J3" s="7" t="inlineStr">
+        <is>
+          <t>Up-to-Date</t>
+        </is>
+      </c>
+      <c r="K3" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="L3" s="9" t="n">
+        <v>9800000</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="11" t="inlineStr">
+        <is>
+          <t>KTA-ACC-02</t>
+        </is>
+      </c>
+      <c r="B4" s="10" t="inlineStr">
+        <is>
+          <t>Palmshore Restaurant Group</t>
+        </is>
+      </c>
+      <c r="C4" s="11" t="inlineStr">
+        <is>
+          <t>Arab-Malabar Fine Dining (5 Outlets)</t>
+        </is>
+      </c>
+      <c r="D4" s="10" t="inlineStr">
+        <is>
+          <t>Chennai, TN</t>
+        </is>
+      </c>
+      <c r="E4" s="10" t="inlineStr">
+        <is>
+          <t>Mr. Faizal</t>
+        </is>
+      </c>
+      <c r="F4" s="11" t="inlineStr">
+        <is>
+          <t>+91 85928 32871</t>
+        </is>
+      </c>
+      <c r="G4" s="12" t="n">
+        <v>850</v>
+      </c>
+      <c r="H4" s="10" t="inlineStr">
+        <is>
+          <t>Green Cardamom 8mm, Dry Ginger, Cloves</t>
+        </is>
+      </c>
+      <c r="I4" s="11" t="inlineStr">
+        <is>
+          <t>15 Days Net</t>
+        </is>
+      </c>
+      <c r="J4" s="11" t="inlineStr">
+        <is>
+          <t>Up-to-Date</t>
+        </is>
+      </c>
+      <c r="K4" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="L4" s="13" t="n">
+        <v>7650000</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="7" t="inlineStr">
+        <is>
+          <t>KTA-ACC-03</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="inlineStr">
+        <is>
+          <t>Dindigul Thalappakatti</t>
+        </is>
+      </c>
+      <c r="C5" s="7" t="inlineStr">
+        <is>
+          <t>Heritage Biryani Chain (45+ Outlets)</t>
+        </is>
+      </c>
+      <c r="D5" s="6" t="inlineStr">
+        <is>
+          <t>South India</t>
+        </is>
+      </c>
+      <c r="E5" s="6" t="inlineStr">
+        <is>
+          <t>Mr. Ramasamy</t>
+        </is>
+      </c>
+      <c r="F5" s="7" t="inlineStr">
+        <is>
+          <t>+91 85928 32871</t>
+        </is>
+      </c>
+      <c r="G5" s="8" t="n">
+        <v>3500</v>
+      </c>
+      <c r="H5" s="6" t="inlineStr">
+        <is>
+          <t>Black Pepper Bold, Cardamom, Cassia</t>
+        </is>
+      </c>
+      <c r="I5" s="7" t="inlineStr">
+        <is>
+          <t>30 Days Net</t>
+        </is>
+      </c>
+      <c r="J5" s="7" t="inlineStr">
+        <is>
+          <t>Current Due</t>
+        </is>
+      </c>
+      <c r="K5" s="9" t="n">
+        <v>425000</v>
+      </c>
+      <c r="L5" s="9" t="n">
+        <v>29400000</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="11" t="inlineStr">
+        <is>
+          <t>KTA-ACC-04</t>
+        </is>
+      </c>
+      <c r="B6" s="10" t="inlineStr">
+        <is>
+          <t>Buhari Restaurant Group (1951)</t>
+        </is>
+      </c>
+      <c r="C6" s="11" t="inlineStr">
+        <is>
+          <t>Heritage Fine Dining (12 Outlets)</t>
+        </is>
+      </c>
+      <c r="D6" s="10" t="inlineStr">
+        <is>
+          <t>Chennai, TN</t>
+        </is>
+      </c>
+      <c r="E6" s="10" t="inlineStr">
+        <is>
+          <t>Mr. Nawaz Buhari</t>
+        </is>
+      </c>
+      <c r="F6" s="11" t="inlineStr">
+        <is>
+          <t>+91 85928 32871</t>
+        </is>
+      </c>
+      <c r="G6" s="12" t="n">
+        <v>1100</v>
+      </c>
+      <c r="H6" s="10" t="inlineStr">
+        <is>
+          <t>Star Anise, Black Pepper, Cloves</t>
+        </is>
+      </c>
+      <c r="I6" s="11" t="inlineStr">
+        <is>
+          <t>15 Days Net</t>
+        </is>
+      </c>
+      <c r="J6" s="11" t="inlineStr">
+        <is>
+          <t>Up-to-Date</t>
+        </is>
+      </c>
+      <c r="K6" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="L6" s="13" t="n">
+        <v>8900000</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="7" t="inlineStr">
+        <is>
+          <t>KTA-ACC-05</t>
+        </is>
+      </c>
+      <c r="B7" s="6" t="inlineStr">
+        <is>
+          <t>Anjappar Chettinad Kitchens</t>
+        </is>
+      </c>
+      <c r="C7" s="7" t="inlineStr">
+        <is>
+          <t>Global Chettinad Brand (30+ Outlets)</t>
+        </is>
+      </c>
+      <c r="D7" s="6" t="inlineStr">
+        <is>
+          <t>Tamil Nadu / KA</t>
+        </is>
+      </c>
+      <c r="E7" s="6" t="inlineStr">
+        <is>
+          <t>Chef Muthukumar</t>
+        </is>
+      </c>
+      <c r="F7" s="7" t="inlineStr">
+        <is>
+          <t>+91 85928 32871</t>
+        </is>
+      </c>
+      <c r="G7" s="8" t="n">
+        <v>2200</v>
+      </c>
+      <c r="H7" s="6" t="inlineStr">
+        <is>
+          <t>Stone Flower (Kalpasi), Star Anise, Jeera</t>
+        </is>
+      </c>
+      <c r="I7" s="7" t="inlineStr">
+        <is>
+          <t>15 Days Net</t>
+        </is>
+      </c>
+      <c r="J7" s="7" t="inlineStr">
+        <is>
+          <t>Up-to-Date</t>
+        </is>
+      </c>
+      <c r="K7" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="L7" s="9" t="n">
+        <v>17600000</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="11" t="inlineStr">
+        <is>
+          <t>KTA-ACC-06</t>
+        </is>
+      </c>
+      <c r="B8" s="10" t="inlineStr">
+        <is>
+          <t>Savya Rasa Culinary Hub</t>
+        </is>
+      </c>
+      <c r="C8" s="11" t="inlineStr">
+        <is>
+          <t>South Indian Luxury Fine Dining</t>
+        </is>
+      </c>
+      <c r="D8" s="10" t="inlineStr">
+        <is>
+          <t>Chennai / Pune</t>
+        </is>
+      </c>
+      <c r="E8" s="10" t="inlineStr">
+        <is>
+          <t>Chef Sheik</t>
+        </is>
+      </c>
+      <c r="F8" s="11" t="inlineStr">
+        <is>
+          <t>+91 85928 32871</t>
+        </is>
+      </c>
+      <c r="G8" s="12" t="n">
+        <v>450</v>
+      </c>
+      <c r="H8" s="10" t="inlineStr">
+        <is>
+          <t>Unbleached Dry Ginger, Royal Star Anise</t>
+        </is>
+      </c>
+      <c r="I8" s="11" t="inlineStr">
+        <is>
+          <t>Immediate NEFT</t>
+        </is>
+      </c>
+      <c r="J8" s="11" t="inlineStr">
+        <is>
+          <t>Up-to-Date</t>
+        </is>
+      </c>
+      <c r="K8" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="L8" s="13" t="n">
+        <v>4200000</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:L1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:K9"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="48" customWidth="1" min="1" max="1"/>
+    <col width="46" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="26" customWidth="1" min="6" max="6"/>
+    <col width="36" customWidth="1" min="7" max="7"/>
+    <col width="27" customWidth="1" min="8" max="8"/>
+    <col width="25" customWidth="1" min="9" max="9"/>
+    <col width="24" customWidth="1" min="10" max="10"/>
+    <col width="26" customWidth="1" min="11" max="11"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>MANNADI WAREHOUSE BATCH INVENTORY LEDGER &amp; LABORATORY QC ASSAY AUDIT</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="5" t="inlineStr">
+        <is>
+          <t>Batch ID</t>
+        </is>
+      </c>
+      <c r="B2" s="5" t="inlineStr">
+        <is>
+          <t>Spice Variety &amp; Grade</t>
+        </is>
+      </c>
+      <c r="C2" s="5" t="inlineStr">
+        <is>
+          <t>HSN Code</t>
+        </is>
+      </c>
+      <c r="D2" s="5" t="inlineStr">
+        <is>
+          <t>Arrival Date</t>
+        </is>
+      </c>
+      <c r="E2" s="5" t="inlineStr">
+        <is>
+          <t>Moisture Assay %</t>
+        </is>
+      </c>
+      <c r="F2" s="5" t="inlineStr">
+        <is>
+          <t>Volatile Oil Retention</t>
+        </is>
+      </c>
+      <c r="G2" s="5" t="inlineStr">
+        <is>
+          <t>Active Assay (Piperine/Curcumin)</t>
+        </is>
+      </c>
+      <c r="H2" s="5" t="inlineStr">
+        <is>
+          <t>Total Stock (40kg Bags)</t>
+        </is>
+      </c>
+      <c r="I2" s="5" t="inlineStr">
+        <is>
+          <t>Available Weight (kg)</t>
+        </is>
+      </c>
+      <c r="J2" s="5" t="inlineStr">
+        <is>
+          <t>Reserved Weight (kg)</t>
+        </is>
+      </c>
+      <c r="K2" s="5" t="inlineStr">
+        <is>
+          <t>Reorder Trigger Status</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="7" t="inlineStr">
+        <is>
+          <t>BATCH-2026-BP01</t>
+        </is>
+      </c>
+      <c r="B3" s="6" t="inlineStr">
+        <is>
+          <t>Black Pepper (Tellicherry TGSEB Bold)</t>
+        </is>
+      </c>
+      <c r="C3" s="7" t="inlineStr">
+        <is>
+          <t>09041140</t>
+        </is>
+      </c>
+      <c r="D3" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="E3" s="7" t="inlineStr">
+        <is>
+          <t>10.4% (&lt;11%)</t>
+        </is>
+      </c>
+      <c r="F3" s="7" t="inlineStr">
+        <is>
+          <t>3.6 ml/100g</t>
+        </is>
+      </c>
+      <c r="G3" s="7" t="inlineStr">
+        <is>
+          <t>6.2% Residual Piperine</t>
+        </is>
+      </c>
+      <c r="H3" s="7" t="n">
+        <v>200</v>
+      </c>
+      <c r="I3" s="8" t="n">
+        <v>8000</v>
+      </c>
+      <c r="J3" s="8" t="n">
+        <v>3500</v>
+      </c>
+      <c r="K3" s="7" t="inlineStr">
+        <is>
+          <t>Optimal Stock</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="11" t="inlineStr">
+        <is>
+          <t>BATCH-2026-GC02</t>
+        </is>
+      </c>
+      <c r="B4" s="10" t="inlineStr">
+        <is>
+          <t>Green Cardamom (Alleppey 8mm+ Extra Bold)</t>
+        </is>
+      </c>
+      <c r="C4" s="11" t="inlineStr">
+        <is>
+          <t>09083140</t>
+        </is>
+      </c>
+      <c r="D4" s="11" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="E4" s="11" t="inlineStr">
+        <is>
+          <t>9.8% (&lt;10%)</t>
+        </is>
+      </c>
+      <c r="F4" s="11" t="inlineStr">
+        <is>
+          <t>8.9 ml/100g</t>
+        </is>
+      </c>
+      <c r="G4" s="11" t="inlineStr">
+        <is>
+          <t>Zero Polish (Natural Green)</t>
+        </is>
+      </c>
+      <c r="H4" s="11" t="n">
+        <v>60</v>
+      </c>
+      <c r="I4" s="12" t="n">
+        <v>1500</v>
+      </c>
+      <c r="J4" s="12" t="n">
+        <v>850</v>
+      </c>
+      <c r="K4" s="11" t="inlineStr">
+        <is>
+          <t>Optimal Stock</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="7" t="inlineStr">
+        <is>
+          <t>BATCH-2026-DG03</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="inlineStr">
+        <is>
+          <t>Unbleached Dry Ginger (Cochin Sun-Dried)</t>
+        </is>
+      </c>
+      <c r="C5" s="7" t="inlineStr">
+        <is>
+          <t>09101110</t>
+        </is>
+      </c>
+      <c r="D5" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="E5" s="7" t="inlineStr">
+        <is>
+          <t>11.1% (&lt;11.5%)</t>
+        </is>
+      </c>
+      <c r="F5" s="7" t="inlineStr">
+        <is>
+          <t>2.4 ml/100g</t>
+        </is>
+      </c>
+      <c r="G5" s="7" t="inlineStr">
+        <is>
+          <t>Zingiberene &gt;3.4%</t>
+        </is>
+      </c>
+      <c r="H5" s="7" t="n">
+        <v>125</v>
+      </c>
+      <c r="I5" s="8" t="n">
+        <v>5000</v>
+      </c>
+      <c r="J5" s="8" t="n">
+        <v>1200</v>
+      </c>
+      <c r="K5" s="7" t="inlineStr">
+        <is>
+          <t>Optimal Stock</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="11" t="inlineStr">
+        <is>
+          <t>BATCH-2026-CL04</t>
+        </is>
+      </c>
+      <c r="B6" s="10" t="inlineStr">
+        <is>
+          <t>Handpicked Whole Cloves (Zanzibar Grade A)</t>
+        </is>
+      </c>
+      <c r="C6" s="11" t="inlineStr">
+        <is>
+          <t>09071010</t>
+        </is>
+      </c>
+      <c r="D6" s="11" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="E6" s="11" t="inlineStr">
+        <is>
+          <t>10.2% (&lt;10.5%)</t>
+        </is>
+      </c>
+      <c r="F6" s="11" t="inlineStr">
+        <is>
+          <t>18.2 ml/100g</t>
+        </is>
+      </c>
+      <c r="G6" s="11" t="inlineStr">
+        <is>
+          <t>Eugenol Retention &gt;92%</t>
+        </is>
+      </c>
+      <c r="H6" s="11" t="n">
+        <v>80</v>
+      </c>
+      <c r="I6" s="12" t="n">
+        <v>3200</v>
+      </c>
+      <c r="J6" s="12" t="n">
+        <v>1600</v>
+      </c>
+      <c r="K6" s="11" t="inlineStr">
+        <is>
+          <t>Optimal Stock</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="7" t="inlineStr">
+        <is>
+          <t>BATCH-2026-SA05</t>
+        </is>
+      </c>
+      <c r="B7" s="6" t="inlineStr">
+        <is>
+          <t>Royal 8-Pointed Star Anise (Annachipoo)</t>
+        </is>
+      </c>
+      <c r="C7" s="7" t="inlineStr">
+        <is>
+          <t>09093100</t>
+        </is>
+      </c>
+      <c r="D7" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="E7" s="7" t="inlineStr">
+        <is>
+          <t>9.5% (&lt;10%)</t>
+        </is>
+      </c>
+      <c r="F7" s="7" t="inlineStr">
+        <is>
+          <t>9.1 ml/100g</t>
+        </is>
+      </c>
+      <c r="G7" s="7" t="inlineStr">
+        <is>
+          <t>Trans-Anethole Active</t>
+        </is>
+      </c>
+      <c r="H7" s="7" t="n">
+        <v>90</v>
+      </c>
+      <c r="I7" s="8" t="n">
+        <v>2250</v>
+      </c>
+      <c r="J7" s="8" t="n">
+        <v>1100</v>
+      </c>
+      <c r="K7" s="7" t="inlineStr">
+        <is>
+          <t>Optimal Stock</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="11" t="inlineStr">
+        <is>
+          <t>BATCH-2026-TM06</t>
+        </is>
+      </c>
+      <c r="B8" s="10" t="inlineStr">
+        <is>
+          <t>Turmeric Powder (Salem High Curcumin)</t>
+        </is>
+      </c>
+      <c r="C8" s="11" t="inlineStr">
+        <is>
+          <t>09103030</t>
+        </is>
+      </c>
+      <c r="D8" s="11" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="E8" s="11" t="inlineStr">
+        <is>
+          <t>9.2% (&lt;10%)</t>
+        </is>
+      </c>
+      <c r="F8" s="11" t="inlineStr">
+        <is>
+          <t>3.8 ml/100g</t>
+        </is>
+      </c>
+      <c r="G8" s="11" t="inlineStr">
+        <is>
+          <t>5.4% Curcumin Content</t>
+        </is>
+      </c>
+      <c r="H8" s="11" t="n">
+        <v>160</v>
+      </c>
+      <c r="I8" s="12" t="n">
+        <v>4000</v>
+      </c>
+      <c r="J8" s="12" t="n">
+        <v>2000</v>
+      </c>
+      <c r="K8" s="11" t="inlineStr">
+        <is>
+          <t>Optimal Stock</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="7" t="inlineStr">
+        <is>
+          <t>BATCH-2026-CS07</t>
+        </is>
+      </c>
+      <c r="B9" s="6" t="inlineStr">
+        <is>
+          <t>Cleaned Whole Cassia Bark Quills</t>
+        </is>
+      </c>
+      <c r="C9" s="7" t="inlineStr">
+        <is>
+          <t>09061190</t>
+        </is>
+      </c>
+      <c r="D9" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="E9" s="7" t="inlineStr">
+        <is>
+          <t>11.4% (&lt;12%)</t>
+        </is>
+      </c>
+      <c r="F9" s="7" t="inlineStr">
+        <is>
+          <t>2.1 ml/100g</t>
+        </is>
+      </c>
+      <c r="G9" s="7" t="inlineStr">
+        <is>
+          <t>Cinnamaldehyde Rich</t>
+        </is>
+      </c>
+      <c r="H9" s="7" t="n">
+        <v>75</v>
+      </c>
+      <c r="I9" s="8" t="n">
+        <v>3000</v>
+      </c>
+      <c r="J9" s="8" t="n">
+        <v>800</v>
+      </c>
+      <c r="K9" s="7" t="inlineStr">
+        <is>
+          <t>Optimal Stock</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:K1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1465,398 +3188,386 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
-    <col width="34" customWidth="1" min="2" max="2"/>
-    <col width="40" customWidth="1" min="3" max="3"/>
-    <col width="22" customWidth="1" min="4" max="4"/>
-    <col width="24" customWidth="1" min="5" max="5"/>
-    <col width="21" customWidth="1" min="6" max="6"/>
+    <col width="17" customWidth="1" min="2" max="2"/>
+    <col width="39" customWidth="1" min="3" max="3"/>
+    <col width="27" customWidth="1" min="4" max="4"/>
+    <col width="38" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
     <col width="19" customWidth="1" min="7" max="7"/>
-    <col width="21" customWidth="1" min="8" max="8"/>
-    <col width="45" customWidth="1" min="9" max="9"/>
+    <col width="24" customWidth="1" min="8" max="8"/>
+    <col width="20" customWidth="1" min="9" max="9"/>
     <col width="36" customWidth="1" min="10" max="10"/>
-    <col width="25" customWidth="1" min="11" max="11"/>
+    <col width="24" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>KEY HOTEL &amp; COMMERCIAL KITCHEN ACCOUNTS DIRECTORY</t>
+          <t>COMMERCIAL INVOICE DISPATCH &amp; LOGISTICS DELIVERY CONFIRMATION LEDGER</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>Account Code</t>
+          <t>Invoice No.</t>
         </is>
       </c>
       <c r="B2" s="5" t="inlineStr">
         <is>
-          <t>Property / Enterprise Name</t>
+          <t>Dispatch Date</t>
         </is>
       </c>
       <c r="C2" s="5" t="inlineStr">
         <is>
-          <t>Establishment Tier</t>
+          <t>Consignee / Client</t>
         </is>
       </c>
       <c r="D2" s="5" t="inlineStr">
         <is>
-          <t>City / Destination</t>
+          <t>Destination Hub</t>
         </is>
       </c>
       <c r="E2" s="5" t="inlineStr">
         <is>
-          <t>Chef / Purchase Lead</t>
+          <t>Items &amp; Varietals</t>
         </is>
       </c>
       <c r="F2" s="5" t="inlineStr">
         <is>
-          <t>Direct Phone Desk</t>
+          <t>Total Bags</t>
         </is>
       </c>
       <c r="G2" s="5" t="inlineStr">
         <is>
-          <t>WhatsApp Desk</t>
+          <t>Net Weight (kg)</t>
         </is>
       </c>
       <c r="H2" s="5" t="inlineStr">
         <is>
-          <t>Monthly Vol. (kg)</t>
+          <t>Invoice Amount (INR)</t>
         </is>
       </c>
       <c r="I2" s="5" t="inlineStr">
         <is>
-          <t>Key SKUs Sourced</t>
+          <t>Payment Mode</t>
         </is>
       </c>
       <c r="J2" s="5" t="inlineStr">
         <is>
-          <t>Logistics SLA</t>
+          <t>Vehicle / Docket ID</t>
         </is>
       </c>
       <c r="K2" s="5" t="inlineStr">
         <is>
-          <t>Annual Run-Rate (INR)</t>
+          <t>Delivery Status</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="7" t="inlineStr">
         <is>
-          <t>KTA-ACC-01</t>
-        </is>
-      </c>
-      <c r="B3" s="6" t="inlineStr">
-        <is>
-          <t>Copper Kitchen Multi-Outlet</t>
-        </is>
-      </c>
-      <c r="C3" s="7" t="inlineStr">
-        <is>
-          <t>Premium Casual Chain (8 Outlets)</t>
+          <t>KTA-INV-2026-40</t>
+        </is>
+      </c>
+      <c r="B3" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="C3" s="6" t="inlineStr">
+        <is>
+          <t>Copper Kitchen Central Commissary</t>
         </is>
       </c>
       <c r="D3" s="6" t="inlineStr">
         <is>
-          <t>Chennai, TN</t>
+          <t>Porur, Chennai</t>
         </is>
       </c>
       <c r="E3" s="6" t="inlineStr">
         <is>
-          <t>Chef Arshad</t>
-        </is>
-      </c>
-      <c r="F3" s="7" t="inlineStr">
-        <is>
-          <t>+91 85928 32871</t>
-        </is>
-      </c>
-      <c r="G3" s="7" t="inlineStr">
-        <is>
-          <t>+91 85928 32871</t>
-        </is>
-      </c>
-      <c r="H3" s="8" t="n">
-        <v>1200</v>
-      </c>
-      <c r="I3" s="6" t="inlineStr">
-        <is>
-          <t>Black Pepper, Kashmiri Chilli, Cloves</t>
+          <t>Black Pepper Bold, Kashmiri Chilli</t>
+        </is>
+      </c>
+      <c r="F3" s="7" t="n">
+        <v>15</v>
+      </c>
+      <c r="G3" s="8" t="n">
+        <v>600</v>
+      </c>
+      <c r="H3" s="9" t="n">
+        <v>450000</v>
+      </c>
+      <c r="I3" s="7" t="inlineStr">
+        <is>
+          <t>15 Days Credit</t>
         </is>
       </c>
       <c r="J3" s="7" t="inlineStr">
         <is>
-          <t>Hotel Smart 24/7 (Same-day)</t>
-        </is>
-      </c>
-      <c r="K3" s="9" t="n">
-        <v>9800000</v>
+          <t>TN-04-AB-8912 (KTA Dedicated)</t>
+        </is>
+      </c>
+      <c r="K3" s="7" t="inlineStr">
+        <is>
+          <t>Delivered &amp; Verified</t>
+        </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="11" t="inlineStr">
         <is>
-          <t>KTA-ACC-02</t>
-        </is>
-      </c>
-      <c r="B4" s="10" t="inlineStr">
-        <is>
-          <t>Palmshore Restaurant Group</t>
-        </is>
-      </c>
-      <c r="C4" s="11" t="inlineStr">
-        <is>
-          <t>Arab-Malabar Fine Dining (5 Outlets)</t>
+          <t>KTA-INV-2026-41</t>
+        </is>
+      </c>
+      <c r="B4" s="11" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="C4" s="10" t="inlineStr">
+        <is>
+          <t>Dindigul Thalappakatti Central Prep</t>
         </is>
       </c>
       <c r="D4" s="10" t="inlineStr">
         <is>
-          <t>Chennai, TN</t>
+          <t>Dindigul Hub</t>
         </is>
       </c>
       <c r="E4" s="10" t="inlineStr">
         <is>
-          <t>Mr. Faizal</t>
-        </is>
-      </c>
-      <c r="F4" s="11" t="inlineStr">
-        <is>
-          <t>+91 85928 32871</t>
-        </is>
-      </c>
-      <c r="G4" s="11" t="inlineStr">
-        <is>
-          <t>+91 85928 32871</t>
-        </is>
-      </c>
-      <c r="H4" s="12" t="n">
-        <v>850</v>
-      </c>
-      <c r="I4" s="10" t="inlineStr">
-        <is>
-          <t>Green Cardamom 8mm, Dry Ginger, Cloves</t>
+          <t>Black Pepper Bold, Cardamom</t>
+        </is>
+      </c>
+      <c r="F4" s="11" t="n">
+        <v>45</v>
+      </c>
+      <c r="G4" s="12" t="n">
+        <v>1800</v>
+      </c>
+      <c r="H4" s="13" t="n">
+        <v>1420000</v>
+      </c>
+      <c r="I4" s="11" t="inlineStr">
+        <is>
+          <t>30 Days Credit</t>
         </is>
       </c>
       <c r="J4" s="11" t="inlineStr">
         <is>
-          <t>Hotel Smart 24/7 (Same-day)</t>
-        </is>
-      </c>
-      <c r="K4" s="13" t="n">
-        <v>7650000</v>
+          <t>TN-57-C-1049 (Express Logistics)</t>
+        </is>
+      </c>
+      <c r="K4" s="11" t="inlineStr">
+        <is>
+          <t>Delivered &amp; Verified</t>
+        </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="7" t="inlineStr">
         <is>
-          <t>KTA-ACC-03</t>
-        </is>
-      </c>
-      <c r="B5" s="6" t="inlineStr">
-        <is>
-          <t>Dindigul Thalappakatti</t>
-        </is>
-      </c>
-      <c r="C5" s="7" t="inlineStr">
-        <is>
-          <t>Heritage Biryani Chain (45+ Outlets)</t>
+          <t>KTA-INV-2026-42</t>
+        </is>
+      </c>
+      <c r="B5" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="C5" s="6" t="inlineStr">
+        <is>
+          <t>Buhari Hotel 1951 Heritage</t>
         </is>
       </c>
       <c r="D5" s="6" t="inlineStr">
         <is>
-          <t>South India</t>
+          <t>Anna Salai, Chennai</t>
         </is>
       </c>
       <c r="E5" s="6" t="inlineStr">
         <is>
-          <t>Mr. Ramasamy</t>
-        </is>
-      </c>
-      <c r="F5" s="7" t="inlineStr">
-        <is>
-          <t>+91 85928 32871</t>
-        </is>
-      </c>
-      <c r="G5" s="7" t="inlineStr">
-        <is>
-          <t>+91 85928 32871</t>
-        </is>
-      </c>
-      <c r="H5" s="8" t="n">
-        <v>3500</v>
-      </c>
-      <c r="I5" s="6" t="inlineStr">
-        <is>
-          <t>Black Pepper Bold, Cardamom, Cassia</t>
+          <t>Star Anise, Whole Cloves, Pepper</t>
+        </is>
+      </c>
+      <c r="F5" s="7" t="n">
+        <v>12</v>
+      </c>
+      <c r="G5" s="8" t="n">
+        <v>480</v>
+      </c>
+      <c r="H5" s="9" t="n">
+        <v>395000</v>
+      </c>
+      <c r="I5" s="7" t="inlineStr">
+        <is>
+          <t>15 Days Credit</t>
         </is>
       </c>
       <c r="J5" s="7" t="inlineStr">
         <is>
-          <t>Bi-Weekly Master Consignments</t>
-        </is>
-      </c>
-      <c r="K5" s="9" t="n">
-        <v>29400000</v>
+          <t>TN-04-AB-8912 (KTA Dedicated)</t>
+        </is>
+      </c>
+      <c r="K5" s="7" t="inlineStr">
+        <is>
+          <t>Delivered &amp; Verified</t>
+        </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="11" t="inlineStr">
         <is>
-          <t>KTA-ACC-04</t>
-        </is>
-      </c>
-      <c r="B6" s="10" t="inlineStr">
-        <is>
-          <t>Buhari Restaurant Group (1951)</t>
-        </is>
-      </c>
-      <c r="C6" s="11" t="inlineStr">
-        <is>
-          <t>Heritage Fine Dining (12 Outlets)</t>
+          <t>KTA-INV-2026-43</t>
+        </is>
+      </c>
+      <c r="B6" s="11" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="C6" s="10" t="inlineStr">
+        <is>
+          <t>Anjappar Chettinad Central</t>
         </is>
       </c>
       <c r="D6" s="10" t="inlineStr">
         <is>
-          <t>Chennai, TN</t>
+          <t>T. Nagar, Chennai</t>
         </is>
       </c>
       <c r="E6" s="10" t="inlineStr">
         <is>
-          <t>Mr. Nawaz Buhari</t>
-        </is>
-      </c>
-      <c r="F6" s="11" t="inlineStr">
-        <is>
-          <t>+91 85928 32871</t>
-        </is>
-      </c>
-      <c r="G6" s="11" t="inlineStr">
-        <is>
-          <t>+91 85928 32871</t>
-        </is>
-      </c>
-      <c r="H6" s="12" t="n">
-        <v>1100</v>
-      </c>
-      <c r="I6" s="10" t="inlineStr">
-        <is>
-          <t>Star Anise, Black Pepper, Cloves</t>
+          <t>Kalpasi, Star Anise, Cumin</t>
+        </is>
+      </c>
+      <c r="F6" s="11" t="n">
+        <v>25</v>
+      </c>
+      <c r="G6" s="12" t="n">
+        <v>1000</v>
+      </c>
+      <c r="H6" s="13" t="n">
+        <v>780000</v>
+      </c>
+      <c r="I6" s="11" t="inlineStr">
+        <is>
+          <t>15 Days Credit</t>
         </is>
       </c>
       <c r="J6" s="11" t="inlineStr">
         <is>
-          <t>Hotel Smart 24/7 (Zero-downtime)</t>
-        </is>
-      </c>
-      <c r="K6" s="13" t="n">
-        <v>8900000</v>
+          <t>TN-04-AB-8912 (KTA Dedicated)</t>
+        </is>
+      </c>
+      <c r="K6" s="11" t="inlineStr">
+        <is>
+          <t>Delivered &amp; Verified</t>
+        </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="7" t="inlineStr">
         <is>
-          <t>KTA-ACC-05</t>
-        </is>
-      </c>
-      <c r="B7" s="6" t="inlineStr">
-        <is>
-          <t>Anjappar Chettinad Kitchens</t>
-        </is>
-      </c>
-      <c r="C7" s="7" t="inlineStr">
-        <is>
-          <t>Global Chettinad Brand (30+ Outlets)</t>
+          <t>KTA-INV-2026-44</t>
+        </is>
+      </c>
+      <c r="B7" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
+      </c>
+      <c r="C7" s="6" t="inlineStr">
+        <is>
+          <t>Palmshore Multi-Outlet Chain</t>
         </is>
       </c>
       <c r="D7" s="6" t="inlineStr">
         <is>
-          <t>Tamil Nadu / KA</t>
+          <t>Ashok Nagar, Chennai</t>
         </is>
       </c>
       <c r="E7" s="6" t="inlineStr">
         <is>
-          <t>Chef Muthukumar</t>
-        </is>
-      </c>
-      <c r="F7" s="7" t="inlineStr">
-        <is>
-          <t>+91 85928 32871</t>
-        </is>
-      </c>
-      <c r="G7" s="7" t="inlineStr">
-        <is>
-          <t>+91 85928 32871</t>
-        </is>
-      </c>
-      <c r="H7" s="8" t="n">
-        <v>2200</v>
-      </c>
-      <c r="I7" s="6" t="inlineStr">
-        <is>
-          <t>Stone Flower (Kalpasi), Star Anise, Jeera</t>
+          <t>Cardamom 8mm, Dry Ginger</t>
+        </is>
+      </c>
+      <c r="F7" s="7" t="n">
+        <v>20</v>
+      </c>
+      <c r="G7" s="8" t="n">
+        <v>800</v>
+      </c>
+      <c r="H7" s="9" t="n">
+        <v>680000</v>
+      </c>
+      <c r="I7" s="7" t="inlineStr">
+        <is>
+          <t>15 Days Credit</t>
         </is>
       </c>
       <c r="J7" s="7" t="inlineStr">
         <is>
-          <t>Weekly Par Replenishment</t>
-        </is>
-      </c>
-      <c r="K7" s="9" t="n">
-        <v>17600000</v>
+          <t>TN-04-AB-8912 (KTA Dedicated)</t>
+        </is>
+      </c>
+      <c r="K7" s="7" t="inlineStr">
+        <is>
+          <t>Delivered &amp; Verified</t>
+        </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="11" t="inlineStr">
         <is>
-          <t>KTA-ACC-06</t>
-        </is>
-      </c>
-      <c r="B8" s="10" t="inlineStr">
-        <is>
-          <t>Savya Rasa Culinary Hub</t>
-        </is>
-      </c>
-      <c r="C8" s="11" t="inlineStr">
-        <is>
-          <t>South Indian Luxury Fine Dining</t>
+          <t>KTA-INV-2026-45</t>
+        </is>
+      </c>
+      <c r="B8" s="11" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="C8" s="10" t="inlineStr">
+        <is>
+          <t>Savya Rasa Fine Dining</t>
         </is>
       </c>
       <c r="D8" s="10" t="inlineStr">
         <is>
-          <t>Chennai / Pune</t>
+          <t>G.N. Chetty Rd, Chennai</t>
         </is>
       </c>
       <c r="E8" s="10" t="inlineStr">
         <is>
-          <t>Chef Sheik</t>
-        </is>
-      </c>
-      <c r="F8" s="11" t="inlineStr">
-        <is>
-          <t>+91 85928 32871</t>
-        </is>
-      </c>
-      <c r="G8" s="11" t="inlineStr">
-        <is>
-          <t>+91 85928 32871</t>
-        </is>
-      </c>
-      <c r="H8" s="12" t="n">
-        <v>450</v>
-      </c>
-      <c r="I8" s="10" t="inlineStr">
-        <is>
-          <t>Unbleached Dry Ginger, Royal Star Anise</t>
+          <t>Unbleached Ginger, Star Anise</t>
+        </is>
+      </c>
+      <c r="F8" s="11" t="n">
+        <v>8</v>
+      </c>
+      <c r="G8" s="12" t="n">
+        <v>320</v>
+      </c>
+      <c r="H8" s="13" t="n">
+        <v>260000</v>
+      </c>
+      <c r="I8" s="11" t="inlineStr">
+        <is>
+          <t>NEFT / Immediate</t>
         </is>
       </c>
       <c r="J8" s="11" t="inlineStr">
         <is>
-          <t>Hotel Smart 24/7 Sourcing</t>
-        </is>
-      </c>
-      <c r="K8" s="13" t="n">
-        <v>4200000</v>
+          <t>TN-04-AB-8912 (KTA Dedicated)</t>
+        </is>
+      </c>
+      <c r="K8" s="11" t="inlineStr">
+        <is>
+          <t>Out for Delivery</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -1867,7 +3578,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2205,245 +3916,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:I6"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="48" customWidth="1" min="1" max="1"/>
-    <col width="48" customWidth="1" min="2" max="2"/>
-    <col width="43" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
-    <col width="17" customWidth="1" min="5" max="5"/>
-    <col width="20" customWidth="1" min="6" max="6"/>
-    <col width="16" customWidth="1" min="7" max="7"/>
-    <col width="18" customWidth="1" min="8" max="8"/>
-    <col width="24" customWidth="1" min="9" max="9"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>WHATSAPP B2B CAMPAIGN &amp; PRO-FORMA CONVERSION LOG</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="5" t="inlineStr">
-        <is>
-          <t>Campaign ID</t>
-        </is>
-      </c>
-      <c r="B2" s="5" t="inlineStr">
-        <is>
-          <t>Campaign Name &amp; Objective</t>
-        </is>
-      </c>
-      <c r="C2" s="5" t="inlineStr">
-        <is>
-          <t>Target Kitchen Segment</t>
-        </is>
-      </c>
-      <c r="D2" s="5" t="inlineStr">
-        <is>
-          <t>Broadcast Date</t>
-        </is>
-      </c>
-      <c r="E2" s="5" t="inlineStr">
-        <is>
-          <t>Messages Sent</t>
-        </is>
-      </c>
-      <c r="F2" s="5" t="inlineStr">
-        <is>
-          <t>Replies Received</t>
-        </is>
-      </c>
-      <c r="G2" s="5" t="inlineStr">
-        <is>
-          <t>Reply Rate %</t>
-        </is>
-      </c>
-      <c r="H2" s="5" t="inlineStr">
-        <is>
-          <t>Qualified RFQs</t>
-        </is>
-      </c>
-      <c r="I2" s="5" t="inlineStr">
-        <is>
-          <t>Closed Revenue (INR)</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="7" t="inlineStr">
-        <is>
-          <t>WA-CAMP-01</t>
-        </is>
-      </c>
-      <c r="B3" s="6" t="inlineStr">
-        <is>
-          <t>Seasonal Flush Green Cardamom 8mm Release</t>
-        </is>
-      </c>
-      <c r="C3" s="6" t="inlineStr">
-        <is>
-          <t>5-Star Hotels &amp; Luxury Banquet Caterers</t>
-        </is>
-      </c>
-      <c r="D3" s="7" t="inlineStr">
-        <is>
-          <t>2026-08-15</t>
-        </is>
-      </c>
-      <c r="E3" s="7" t="n">
-        <v>250</v>
-      </c>
-      <c r="F3" s="7" t="n">
-        <v>94</v>
-      </c>
-      <c r="G3" s="7" t="inlineStr">
-        <is>
-          <t>37.6%</t>
-        </is>
-      </c>
-      <c r="H3" s="7" t="n">
-        <v>28</v>
-      </c>
-      <c r="I3" s="9" t="n">
-        <v>2450000</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="11" t="inlineStr">
-        <is>
-          <t>WA-CAMP-02</t>
-        </is>
-      </c>
-      <c r="B4" s="10" t="inlineStr">
-        <is>
-          <t>Hotel Smart 24/7 Zero-Downtime Restock</t>
-        </is>
-      </c>
-      <c r="C4" s="10" t="inlineStr">
-        <is>
-          <t>Chennai Multi-Outlet Restaurant Chains</t>
-        </is>
-      </c>
-      <c r="D4" s="11" t="inlineStr">
-        <is>
-          <t>2026-08-20</t>
-        </is>
-      </c>
-      <c r="E4" s="11" t="n">
-        <v>380</v>
-      </c>
-      <c r="F4" s="11" t="n">
-        <v>142</v>
-      </c>
-      <c r="G4" s="11" t="inlineStr">
-        <is>
-          <t>37.4%</t>
-        </is>
-      </c>
-      <c r="H4" s="11" t="n">
-        <v>45</v>
-      </c>
-      <c r="I4" s="13" t="n">
-        <v>4820000</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="7" t="inlineStr">
-        <is>
-          <t>WA-CAMP-03</t>
-        </is>
-      </c>
-      <c r="B5" s="6" t="inlineStr">
-        <is>
-          <t>Tellicherry Black Pepper TGSEB Export Lot</t>
-        </is>
-      </c>
-      <c r="C5" s="6" t="inlineStr">
-        <is>
-          <t>Cloud Kitchen Commissaries &amp; Exporters</t>
-        </is>
-      </c>
-      <c r="D5" s="7" t="inlineStr">
-        <is>
-          <t>2026-08-25</t>
-        </is>
-      </c>
-      <c r="E5" s="7" t="n">
-        <v>190</v>
-      </c>
-      <c r="F5" s="7" t="n">
-        <v>78</v>
-      </c>
-      <c r="G5" s="7" t="inlineStr">
-        <is>
-          <t>41.1%</t>
-        </is>
-      </c>
-      <c r="H5" s="7" t="n">
-        <v>22</v>
-      </c>
-      <c r="I5" s="9" t="n">
-        <v>3120000</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="11" t="inlineStr">
-        <is>
-          <t>WA-CAMP-04</t>
-        </is>
-      </c>
-      <c r="B6" s="10" t="inlineStr">
-        <is>
-          <t>Chef Welcome Box Complimentary Discovery Trial</t>
-        </is>
-      </c>
-      <c r="C6" s="10" t="inlineStr">
-        <is>
-          <t>Executive Chefs in TN &amp; Bangalore</t>
-        </is>
-      </c>
-      <c r="D6" s="11" t="inlineStr">
-        <is>
-          <t>2026-08-28</t>
-        </is>
-      </c>
-      <c r="E6" s="11" t="n">
-        <v>320</v>
-      </c>
-      <c r="F6" s="11" t="n">
-        <v>168</v>
-      </c>
-      <c r="G6" s="11" t="inlineStr">
-        <is>
-          <t>52.5%</t>
-        </is>
-      </c>
-      <c r="H6" s="11" t="n">
-        <v>64</v>
-      </c>
-      <c r="I6" s="13" t="n">
-        <v>5900000</v>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A1:I1"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>